<commit_message>
docs: update hardware BOM
</commit_message>
<xml_diff>
--- a/hardware/BOM_magicKey.xlsx
+++ b/hardware/BOM_magicKey.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7967DFA2-E267-4063-900E-0759BB59B995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D60DF2-9058-49DC-8A4E-535990581094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27240" yWindow="2445" windowWidth="39780" windowHeight="18180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34995" yWindow="675" windowWidth="39780" windowHeight="18180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_magicKeySCH_magicKeySCH_202" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="125">
   <si>
     <t>No.</t>
   </si>
@@ -50,9 +50,6 @@
   </si>
   <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>KEY-PB8</t>
   </si>
   <si>
     <t>A1,A2,A3,A4,A5,A6,A7,A8,A9,A10,A11,A12,A13,A14,A15,A16,A17,A18,A19,A20,A21,A22,A23,A24,A25,A26,A27,A28,A29,A30,A31,A32,A33,A34,A35,A36,A37,A38,A39,A40,A41,A42,A43,A44,A45,A46,A47,A48,A49,A50,A51,A52,A53,A54,A55,A56,A57,A58,A59,A60,A61,A62,A63</t>
@@ -390,6 +387,14 @@
   </si>
   <si>
     <t>U6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KEY-PB8</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -777,7 +782,8 @@
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="4" width="20" customWidth="1"/>
+    <col min="1" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="29.125" customWidth="1"/>
     <col min="5" max="5" width="50.375" customWidth="1"/>
     <col min="6" max="10" width="20" customWidth="1"/>
   </cols>
@@ -822,673 +828,673 @@
         <v>63</v>
       </c>
       <c r="C2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
       <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>30</v>
       </c>
       <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
         <v>26</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>27</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" t="s">
         <v>28</v>
       </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>29</v>
       </c>
-      <c r="I6" t="s">
-        <v>30</v>
-      </c>
       <c r="J6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B7">
         <v>9</v>
       </c>
       <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
         <v>32</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
         <v>34</v>
       </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>35</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>36</v>
       </c>
-      <c r="I7" t="s">
-        <v>37</v>
-      </c>
       <c r="J7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
         <v>39</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>40</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" t="s">
         <v>41</v>
       </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s">
-        <v>39</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>42</v>
       </c>
-      <c r="I8" t="s">
-        <v>43</v>
-      </c>
       <c r="J8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
         <v>45</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>46</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" t="s">
         <v>47</v>
       </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>48</v>
       </c>
-      <c r="I9" t="s">
-        <v>49</v>
-      </c>
       <c r="J9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" t="s">
         <v>54</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>55</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" t="s">
         <v>56</v>
       </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s">
-        <v>54</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>57</v>
       </c>
-      <c r="I10" t="s">
-        <v>58</v>
-      </c>
       <c r="J10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
       <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
         <v>60</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>61</v>
       </c>
-      <c r="E11" t="s">
-        <v>62</v>
-      </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" t="s">
         <v>64</v>
       </c>
-      <c r="D12" t="s">
-        <v>65</v>
-      </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B13">
         <v>3</v>
       </c>
       <c r="C13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" t="s">
         <v>67</v>
       </c>
-      <c r="D13" t="s">
-        <v>68</v>
-      </c>
       <c r="E13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" t="s">
         <v>70</v>
       </c>
-      <c r="D14" t="s">
-        <v>71</v>
-      </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B16">
         <v>63</v>
       </c>
       <c r="C16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" t="s">
         <v>75</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>76</v>
       </c>
-      <c r="E16" t="s">
-        <v>77</v>
-      </c>
       <c r="F16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" t="s">
+        <v>78</v>
+      </c>
+      <c r="D17" t="s">
         <v>79</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>80</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" t="s">
+        <v>78</v>
+      </c>
+      <c r="H17" t="s">
         <v>81</v>
       </c>
-      <c r="F17" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" t="s">
-        <v>79</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>82</v>
       </c>
-      <c r="I17" t="s">
-        <v>83</v>
-      </c>
       <c r="J17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" t="s">
         <v>85</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>86</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" t="s">
         <v>87</v>
       </c>
-      <c r="F18" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" t="s">
-        <v>85</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>88</v>
       </c>
-      <c r="I18" t="s">
-        <v>89</v>
-      </c>
       <c r="J18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" t="s">
         <v>91</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>92</v>
       </c>
-      <c r="E19" t="s">
-        <v>93</v>
-      </c>
       <c r="F19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" t="s">
         <v>95</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>96</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" t="s">
+        <v>94</v>
+      </c>
+      <c r="H20" t="s">
         <v>97</v>
       </c>
-      <c r="F20" t="s">
-        <v>14</v>
-      </c>
-      <c r="G20" t="s">
-        <v>95</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>98</v>
       </c>
-      <c r="I20" t="s">
-        <v>99</v>
-      </c>
       <c r="J20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" t="s">
+        <v>122</v>
+      </c>
+      <c r="E21" t="s">
         <v>101</v>
       </c>
-      <c r="D21" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" t="s">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
         <v>102</v>
       </c>
-      <c r="F21" t="s">
-        <v>14</v>
-      </c>
-      <c r="G21" t="s">
-        <v>101</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="I21" t="s">
-        <v>104</v>
-      </c>
       <c r="J21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
+        <v>105</v>
+      </c>
+      <c r="D22" t="s">
         <v>106</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>107</v>
       </c>
-      <c r="E22" t="s">
-        <v>108</v>
-      </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1547,33 +1553,33 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" t="s">
         <v>48</v>
       </c>
-      <c r="I2" t="s">
-        <v>49</v>
-      </c>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1628,101 +1634,101 @@
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2">
-        <v>1</v>
+      <c r="B2" t="s">
+        <v>123</v>
       </c>
       <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>51</v>
       </c>
-      <c r="E2" t="s">
-        <v>52</v>
-      </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" t="s">
         <v>119</v>
       </c>
-      <c r="D3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E3" t="s">
-        <v>120</v>
-      </c>
       <c r="F3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" t="s">
         <v>113</v>
       </c>
-      <c r="D4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" t="s">
-        <v>114</v>
-      </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>